<commit_message>
Update: New Constraints added
</commit_message>
<xml_diff>
--- a/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
+++ b/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
@@ -5,26 +5,40 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krdes\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23702518-2386-494F-9118-62E95892C467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9515303A-490A-4EFB-9521-8627113563E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="651" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="651" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controller_Limits" sheetId="1" r:id="rId1"/>
-    <sheet name="IO_Module_Catalog" sheetId="2" r:id="rId2"/>
-    <sheet name="NIO_System_Constraints" sheetId="3" r:id="rId3"/>
-    <sheet name="NIO_Ambient_Current_Limits" sheetId="4" r:id="rId4"/>
-    <sheet name="Project_IO" sheetId="5" r:id="rId5"/>
+    <sheet name="Mounting Rule" sheetId="6" r:id="rId2"/>
+    <sheet name="IO_Module_Catalog" sheetId="2" r:id="rId3"/>
+    <sheet name="NIO_System_Constraints" sheetId="3" r:id="rId4"/>
+    <sheet name="NIO_Ambient_Current_Limits" sheetId="4" r:id="rId5"/>
+    <sheet name="Project_IO" sheetId="5" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="127">
   <si>
     <t>Controller_Model</t>
   </si>
@@ -375,18 +389,54 @@
   </si>
   <si>
     <t>Redundancy</t>
+  </si>
+  <si>
+    <t>Node Type</t>
+  </si>
+  <si>
+    <t>SNU</t>
+  </si>
+  <si>
+    <t>IOM</t>
+  </si>
+  <si>
+    <t>SSB401</t>
+  </si>
+  <si>
+    <t>SPW48_</t>
+  </si>
+  <si>
+    <t>SCU_Without_ESB</t>
+  </si>
+  <si>
+    <t>SCU_With_ESB</t>
+  </si>
+  <si>
+    <t>SEC40_</t>
+  </si>
+  <si>
+    <t>Slot</t>
+  </si>
+  <si>
+    <t>Type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -404,7 +454,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -412,13 +462,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -939,10 +1010,430 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C680BE8D-D222-4E6F-9A6F-956488FCAF86}">
+  <dimension ref="A1:C37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="2">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="2">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" s="2">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="2">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="2">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="2">
+        <v>11</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" s="2">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="2">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" s="2">
+        <v>3</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" s="2">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B18" s="2">
+        <v>5</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" s="2">
+        <v>6</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="2">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="2">
+        <v>8</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" s="2">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="2">
+        <v>10</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="2">
+        <v>11</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="2">
+        <v>12</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" s="2">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="2">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" s="2">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" s="2">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" s="2">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" s="2">
+        <v>6</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B32" s="2">
+        <v>7</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" s="2">
+        <v>8</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B34" s="2">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" s="2">
+        <v>10</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B36" s="2">
+        <v>11</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" s="2">
+        <v>12</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2298,7 +2789,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2397,7 +2888,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2467,7 +2958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Fix: Clean folder structure
</commit_message>
<xml_diff>
--- a/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
+++ b/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFDAA91-7DB0-4845-A2D7-DE01F2F5B59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF44EA6A-52FD-47F1-B48F-AA90C97A8C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72" yWindow="1032" windowWidth="15636" windowHeight="10668" tabRatio="781" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="781" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controller_Limits" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="IO_Module_Catalog" sheetId="2" r:id="rId3"/>
     <sheet name="NIO_System_Constraints" sheetId="3" r:id="rId4"/>
     <sheet name="NIO_Ambient_Current_Limits" sheetId="4" r:id="rId5"/>
-    <sheet name="Project_IO" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="124">
   <si>
     <t>Controller_Model</t>
   </si>
@@ -376,18 +375,6 @@
     <t>Max_Total_Current_A</t>
   </si>
   <si>
-    <t>System</t>
-  </si>
-  <si>
-    <t>Required_Channels</t>
-  </si>
-  <si>
-    <t>Ambient_C</t>
-  </si>
-  <si>
-    <t>Redundancy</t>
-  </si>
-  <si>
     <t>Node Type</t>
   </si>
   <si>
@@ -419,6 +406,9 @@
   </si>
   <si>
     <t>AI, DI, DO, AO</t>
+  </si>
+  <si>
+    <t>SPW482</t>
   </si>
 </sst>
 </file>
@@ -1025,227 +1015,227 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B3" s="2">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B5" s="2">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B7" s="2">
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B8" s="2">
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B9" s="2">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B10" s="2">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B11" s="2">
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B13" s="2">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B15" s="2">
         <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B16" s="2">
         <v>3</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B17" s="2">
         <v>4</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B19" s="2">
         <v>6</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B20" s="2">
         <v>7</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B21" s="2">
         <v>8</v>
@@ -1254,178 +1244,178 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B22" s="2">
         <v>9</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B23" s="2">
         <v>10</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B24" s="2">
         <v>11</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>120</v>
+      <c r="C24" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B25" s="2">
         <v>12</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>120</v>
+      <c r="C25" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B26" s="2">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B27" s="2">
         <v>2</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B28" s="2">
         <v>3</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B29" s="2">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B31" s="2">
         <v>6</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B32" s="2">
         <v>7</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B33" s="2">
         <v>8</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B34" s="2">
         <v>9</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B35" s="2">
         <v>10</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B36" s="2">
         <v>11</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>120</v>
+      <c r="C36" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B37" s="2">
         <v>12</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>120</v>
+      <c r="C37" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2477,7 +2467,7 @@
         <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D17" t="s">
         <v>73</v>
@@ -2957,54 +2947,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" t="s">
-        <v>113</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" t="s">
-        <v>114</v>
-      </c>
-      <c r="I1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
update: test cases added
</commit_message>
<xml_diff>
--- a/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
+++ b/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF44EA6A-52FD-47F1-B48F-AA90C97A8C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BB4CFD-2593-4EEA-A4F4-C221AF508001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="781" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="781" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controller_Limits" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,10 @@
     <sheet name="NIO_System_Constraints" sheetId="3" r:id="rId4"/>
     <sheet name="NIO_Ambient_Current_Limits" sheetId="4" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Controller_Limits!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">IO_Module_Catalog!$A$1:$U$21</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="126">
   <si>
     <t>Controller_Model</t>
   </si>
@@ -387,18 +391,12 @@
     <t>SSB401</t>
   </si>
   <si>
-    <t>SPW48_</t>
-  </si>
-  <si>
     <t>SCU_Without_ESB</t>
   </si>
   <si>
     <t>SCU_With_ESB</t>
   </si>
   <si>
-    <t>SEC40_</t>
-  </si>
-  <si>
     <t>Slot</t>
   </si>
   <si>
@@ -409,6 +407,18 @@
   </si>
   <si>
     <t>SPW482</t>
+  </si>
+  <si>
+    <t>SEC401</t>
+  </si>
+  <si>
+    <t>Node No</t>
+  </si>
+  <si>
+    <t>Node 1 Only</t>
+  </si>
+  <si>
+    <t>&gt;1</t>
   </si>
 </sst>
 </file>
@@ -424,9 +434,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -473,11 +485,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -785,220 +799,222 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>32</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="1">
         <v>108</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="3">
         <v>13</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="3">
         <v>110</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="3">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>32</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>108</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="3">
         <v>13</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="3">
         <v>110</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="3">
         <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
         <v>13</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="1">
         <v>110</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="1">
         <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
         <v>13</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="1">
         <v>110</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="1">
         <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
         <v>9</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <v>78</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="1">
         <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
         <v>9</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="1">
         <v>78</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="1">
         <v>39</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1006,416 +1022,528 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C680BE8D-D222-4E6F-9A6F-956488FCAF86}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="1">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="1">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="1">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" s="1">
+        <v>8</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="1">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="1">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="1">
+        <v>11</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B13" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" s="1">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" s="1">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" s="1">
         <v>6</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D19" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="1">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D20" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="1">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D21" s="1"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="1">
+        <v>9</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="1">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="1">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="1">
+        <v>12</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="1">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B10" s="2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="1">
+        <v>1</v>
+      </c>
+      <c r="C28" s="1">
+        <v>3</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="1">
+        <v>1</v>
+      </c>
+      <c r="C29" s="1">
+        <v>4</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" s="1">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1">
+        <v>5</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" s="1">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1">
+        <v>6</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="1">
+        <v>1</v>
+      </c>
+      <c r="C32" s="1">
+        <v>7</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="1">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1">
+        <v>8</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+      <c r="C34" s="1">
         <v>9</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D34" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B11" s="2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B35" s="1">
+        <v>1</v>
+      </c>
+      <c r="C35" s="1">
         <v>10</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D35" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B36" s="1">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1">
         <v>11</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="D36" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1">
         <v>12</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="2">
-        <v>1</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B15" s="2">
-        <v>2</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B16" s="2">
-        <v>3</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B17" s="2">
-        <v>4</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B18" s="2">
-        <v>5</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B19" s="2">
-        <v>6</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B20" s="2">
-        <v>7</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" s="2">
-        <v>8</v>
-      </c>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="2">
-        <v>9</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B23" s="2">
-        <v>10</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="2">
-        <v>11</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B25" s="2">
-        <v>12</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26" s="2">
-        <v>1</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B27" s="2">
-        <v>2</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B28" s="2">
-        <v>3</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B29" s="2">
-        <v>4</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B30" s="2">
-        <v>5</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31" s="2">
-        <v>6</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B32" s="2">
-        <v>7</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" s="2">
-        <v>8</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B34" s="2">
-        <v>9</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B35" s="2">
-        <v>10</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B36" s="2">
-        <v>11</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B37" s="2">
-        <v>12</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>123</v>
+      <c r="D37" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1429,1353 +1557,1365 @@
   <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="62.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.21875" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" customWidth="1"/>
+    <col min="7" max="7" width="64.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.21875" customWidth="1"/>
+    <col min="17" max="17" width="21.88671875" customWidth="1"/>
+    <col min="18" max="18" width="17.109375" customWidth="1"/>
+    <col min="19" max="19" width="17.5546875" customWidth="1"/>
+    <col min="20" max="20" width="29.77734375" customWidth="1"/>
+    <col min="21" max="21" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="1">
         <v>60</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="1">
         <v>16</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="1">
         <v>3</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="1">
         <v>5</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="1">
         <v>22</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="1">
         <v>25</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P2" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q2" t="s">
+      <c r="P2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R2" t="s">
-        <v>46</v>
-      </c>
-      <c r="S2" t="s">
+      <c r="R2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="1">
         <v>65</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="1">
         <v>14</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="1">
         <v>3</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="1">
         <v>5</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="1">
         <v>22</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="1">
         <v>25</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P3" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="P3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R3" t="s">
-        <v>46</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="R3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>16</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="1">
         <v>70</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="1">
         <v>10</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="1">
         <v>3</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="1">
         <v>5</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="1">
         <v>22</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="1">
         <v>25</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="P4" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q4" t="s">
+      <c r="P4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R4" t="s">
-        <v>46</v>
-      </c>
-      <c r="S4" t="s">
+      <c r="R4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="U4" t="s">
+      <c r="U4" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>16</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="1">
         <v>65</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="1">
         <v>16</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="1">
         <v>5</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="1">
         <v>4</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="1">
         <v>7</v>
       </c>
-      <c r="P5" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q5" t="s">
+      <c r="O5" s="1"/>
+      <c r="P5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R5" t="s">
-        <v>46</v>
-      </c>
-      <c r="S5" t="s">
+      <c r="R5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T5" t="s">
+      <c r="T5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="U5" t="s">
+      <c r="U5" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>16</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="1">
         <v>70</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="1">
         <v>12</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="1">
         <v>3</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="1">
         <v>5</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="1">
         <v>4</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="1">
         <v>7</v>
       </c>
-      <c r="P6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q6" t="s">
+      <c r="O6" s="1"/>
+      <c r="P6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R6" t="s">
-        <v>46</v>
-      </c>
-      <c r="S6" t="s">
+      <c r="R6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S6" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T6" t="s">
+      <c r="T6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="U6" t="s">
+      <c r="U6" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>16</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="1">
         <v>60</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="1">
         <v>16</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="1">
         <v>3</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="1">
         <v>6</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="1">
         <v>25</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="1">
         <v>29</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="P7" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q7" t="s">
+      <c r="P7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R7" t="s">
-        <v>46</v>
-      </c>
-      <c r="S7" t="s">
+      <c r="R7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T7" t="s">
+      <c r="T7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U7" t="s">
+      <c r="U7" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>16</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="1">
         <v>65</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="1">
         <v>14</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="1">
         <v>3</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="1">
         <v>6</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="1">
         <v>25</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="1">
         <v>29</v>
       </c>
-      <c r="P8" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q8" t="s">
+      <c r="O8" s="1"/>
+      <c r="P8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R8" t="s">
-        <v>46</v>
-      </c>
-      <c r="S8" t="s">
+      <c r="R8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T8" t="s">
+      <c r="T8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U8" t="s">
+      <c r="U8" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="1">
         <v>16</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="1">
         <v>70</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="1">
         <v>8</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="1">
         <v>3</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="1">
         <v>6</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="1">
         <v>25</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="1">
         <v>29</v>
       </c>
-      <c r="P9" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q9" t="s">
+      <c r="O9" s="1"/>
+      <c r="P9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R9" t="s">
-        <v>46</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="R9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T9" t="s">
+      <c r="T9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U9" t="s">
+      <c r="U9" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="1">
         <v>16</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="1">
         <v>65</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="1">
         <v>16</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="1">
         <v>3</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="1">
         <v>6</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="1">
         <v>5</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="1">
         <v>10</v>
       </c>
-      <c r="P10" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="O10" s="1"/>
+      <c r="P10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S10" t="s">
+      <c r="R10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T10" t="s">
+      <c r="T10" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U10" t="s">
+      <c r="U10" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="1">
         <v>16</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="1">
         <v>70</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="1">
         <v>12</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="1">
         <v>3</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="1">
         <v>6</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="1">
         <v>5</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="1">
         <v>10</v>
       </c>
-      <c r="P11" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="O11" s="1"/>
+      <c r="P11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R11" t="s">
-        <v>46</v>
-      </c>
-      <c r="S11" t="s">
+      <c r="R11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T11" t="s">
+      <c r="T11" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="U11" t="s">
+      <c r="U11" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="1">
         <v>16</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="1">
         <v>65</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="1">
         <v>16</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="1">
         <v>2</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="1">
         <v>4</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="1">
         <v>2</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="1">
         <v>4</v>
       </c>
-      <c r="P12" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q12" t="s">
+      <c r="O12" s="1"/>
+      <c r="P12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R12" t="s">
-        <v>46</v>
-      </c>
-      <c r="S12" t="s">
+      <c r="R12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T12" t="s">
+      <c r="T12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U12" t="s">
+      <c r="U12" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="1">
         <v>16</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="1">
         <v>70</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="1">
         <v>12</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="1">
         <v>2</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="1">
         <v>4</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="1">
         <v>2</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="1">
         <v>4</v>
       </c>
-      <c r="P13" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q13" t="s">
+      <c r="O13" s="1"/>
+      <c r="P13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R13" t="s">
-        <v>46</v>
-      </c>
-      <c r="S13" t="s">
+      <c r="R13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S13" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T13" t="s">
+      <c r="T13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U13" t="s">
+      <c r="U13" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="1">
         <v>16</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="1">
         <v>60</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="1">
         <v>16</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="1">
         <v>3</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="1">
         <v>6</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="1">
         <v>5</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="1">
         <v>7</v>
       </c>
-      <c r="P14" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q14" t="s">
+      <c r="O14" s="1"/>
+      <c r="P14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R14" t="s">
-        <v>46</v>
-      </c>
-      <c r="S14" t="s">
+      <c r="R14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T14" t="s">
+      <c r="T14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="U14" t="s">
+      <c r="U14" s="1" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="1">
         <v>16</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="1">
         <v>65</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="1">
         <v>12</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="1">
         <v>3</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="1">
         <v>6</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="1">
         <v>5</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="1">
         <v>7</v>
       </c>
-      <c r="P15" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q15" t="s">
+      <c r="O15" s="1"/>
+      <c r="P15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q15" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R15" t="s">
-        <v>46</v>
-      </c>
-      <c r="S15" t="s">
+      <c r="R15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T15" t="s">
+      <c r="T15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="U15" t="s">
+      <c r="U15" s="1" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="1">
         <v>16</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="1">
         <v>70</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="1">
         <v>10</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="1">
         <v>3</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="1">
         <v>6</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="1">
         <v>5</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="1">
         <v>7</v>
       </c>
-      <c r="P16" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="O16" s="1"/>
+      <c r="P16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R16" t="s">
-        <v>46</v>
-      </c>
-      <c r="S16" t="s">
+      <c r="R16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T16" t="s">
+      <c r="T16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="U16" t="s">
+      <c r="U16" s="1" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C17" t="s">
-        <v>122</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>16</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="1">
         <v>70</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="1">
         <v>16</v>
       </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>0</v>
-      </c>
-      <c r="O17" t="s">
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>0</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="P17" t="s">
+      <c r="P17" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="Q17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R17" t="s">
-        <v>46</v>
-      </c>
-      <c r="S17" t="s">
+      <c r="R17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T17" t="s">
+      <c r="T17" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="U17" t="s">
+      <c r="U17" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="1">
         <v>16</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="1">
         <v>70</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="1">
         <v>16</v>
       </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>0</v>
-      </c>
-      <c r="O18" t="s">
+      <c r="K18" s="1">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="N18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="P18" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q18" t="s">
+      <c r="P18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R18" t="s">
-        <v>46</v>
-      </c>
-      <c r="S18" t="s">
+      <c r="R18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S18" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T18" t="s">
+      <c r="T18" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="U18" t="s">
+      <c r="U18" s="1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="1">
         <v>70</v>
       </c>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>0</v>
-      </c>
-      <c r="P19" t="s">
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="Q19" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R19" t="s">
-        <v>46</v>
-      </c>
-      <c r="S19" t="s">
+      <c r="R19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S19" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T19" t="s">
+      <c r="T19" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="U19" t="s">
+      <c r="U19" s="1" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="1">
         <v>70</v>
       </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="P20" t="s">
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="Q20" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R20" t="s">
-        <v>46</v>
-      </c>
-      <c r="S20" t="s">
+      <c r="R20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T20" t="s">
+      <c r="T20" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="U20" t="s">
+      <c r="U20" s="1" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="1">
         <v>70</v>
       </c>
-      <c r="J21">
-        <v>0</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <v>0</v>
-      </c>
-      <c r="P21" t="s">
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1">
+        <v>0</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="Q21" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="R21" t="s">
-        <v>46</v>
-      </c>
-      <c r="S21" t="s">
+      <c r="R21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S21" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="T21" t="s">
+      <c r="T21" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="U21" t="s">
+      <c r="U21" s="1" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U21" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
update: Domain logic updated to use pandas df
</commit_message>
<xml_diff>
--- a/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
+++ b/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECEFC95-CF49-43BB-B63D-409469EDBDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E561AC05-0409-491E-B9FA-485E225FAE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8004" yWindow="1260" windowWidth="13608" windowHeight="9648" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="127">
   <si>
     <t>Controller_Model</t>
   </si>
@@ -421,6 +421,9 @@
   </si>
   <si>
     <t>&gt;=2</t>
+  </si>
+  <si>
+    <t>Empty</t>
   </si>
 </sst>
 </file>
@@ -1503,7 +1506,9 @@
       <c r="C33" s="1">
         <v>8</v>
       </c>
-      <c r="D33" s="1"/>
+      <c r="D33" s="1" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">

</xml_diff>

<commit_message>
update: Bill of material added
</commit_message>
<xml_diff>
--- a/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
+++ b/templates/Yokogawa_SIS_Constraints_Model_v3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E561AC05-0409-491E-B9FA-485E225FAE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BC2BDB-F2E1-4F97-AE0F-2E25C18B0C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8004" yWindow="1260" windowWidth="13608" windowHeight="9648" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="781" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controller_Limits" sheetId="1" r:id="rId1"/>
@@ -2947,7 +2947,7 @@
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>

</xml_diff>